<commit_message>
fix: remove FINAL.xlsx spreadsheet from repository
</commit_message>
<xml_diff>
--- a/FINAL.xlsx
+++ b/FINAL.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Lenovo\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Lenovo\bagi-hasil\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0968BC88-8C7D-4CAA-BB7C-FAA9F616E5F7}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A3E5AE62-8701-4ED0-A08B-1814EE8E995C}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="122" uniqueCount="81">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="132" uniqueCount="81">
   <si>
     <t>ABDUL MUNAJAT</t>
   </si>
@@ -1127,7 +1127,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:AG100"/>
+  <dimension ref="A1:AG102"/>
   <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="28" customWidth="1"/>
@@ -1416,7 +1416,7 @@
         <v>40400000</v>
       </c>
       <c r="J5" s="12">
-        <f t="shared" ref="J5:J12" si="0">D5*$J$3</f>
+        <f t="shared" ref="J5:J14" si="0">D5*$J$3</f>
         <v>2968800</v>
       </c>
       <c r="K5" s="12">
@@ -1428,23 +1428,23 @@
         <v>1255040</v>
       </c>
       <c r="M5" s="12">
-        <f t="shared" ref="M5:M12" si="1">G5*$M$3</f>
+        <f t="shared" ref="M5:M14" si="1">G5*$M$3</f>
         <v>0</v>
       </c>
       <c r="N5" s="12">
-        <f t="shared" ref="N5:N12" si="2">H5*$N$3</f>
+        <f t="shared" ref="N5:N14" si="2">H5*$N$3</f>
         <v>105000</v>
       </c>
       <c r="O5" s="12">
-        <f t="shared" ref="O5:O12" si="3">SUM(J5:N5)</f>
+        <f t="shared" ref="O5:O14" si="3">SUM(J5:N5)</f>
         <v>10714040</v>
       </c>
       <c r="P5" s="12">
-        <f t="shared" ref="P5:P12" si="4">I5*30%</f>
+        <f t="shared" ref="P5:P14" si="4">I5*30%</f>
         <v>12120000</v>
       </c>
       <c r="Q5" s="12">
-        <f t="shared" ref="Q5:Q12" si="5">O5-P5</f>
+        <f t="shared" ref="Q5:Q14" si="5">O5-P5</f>
         <v>-1405960</v>
       </c>
       <c r="R5" s="13">
@@ -1462,20 +1462,20 @@
         <v>100000</v>
       </c>
       <c r="AB5" s="12">
-        <f t="shared" ref="AB5:AB12" si="6">SUM(S5:AA5)</f>
+        <f t="shared" ref="AB5:AB14" si="6">SUM(S5:AA5)</f>
         <v>100000</v>
       </c>
       <c r="AC5" s="12">
         <v>0</v>
       </c>
       <c r="AD5" s="12">
-        <f t="shared" ref="AD5:AD12" si="7">O5-AB5</f>
+        <f t="shared" ref="AD5:AD14" si="7">O5-AB5</f>
         <v>10614040</v>
       </c>
       <c r="AE5" s="14"/>
       <c r="AF5" s="14"/>
       <c r="AG5" s="12">
-        <f t="shared" ref="AG5:AG12" si="8">AE5+AF5</f>
+        <f t="shared" ref="AG5:AG14" si="8">AE5+AF5</f>
         <v>0</v>
       </c>
     </row>
@@ -1606,11 +1606,11 @@
         <v>2651400</v>
       </c>
       <c r="K7" s="12">
-        <f t="shared" ref="K7:K12" si="9">E7*$K$3</f>
+        <f t="shared" ref="K7:K14" si="9">E7*$K$3</f>
         <v>2586000</v>
       </c>
       <c r="L7" s="12">
-        <f t="shared" ref="L7:L12" si="10">F7*$L$3</f>
+        <f t="shared" ref="L7:L14" si="10">F7*$L$3</f>
         <v>3027840</v>
       </c>
       <c r="M7" s="12">
@@ -1989,35 +1989,35 @@
         <v>331000</v>
       </c>
       <c r="J11" s="12">
-        <f t="shared" si="0"/>
+        <f t="shared" ref="J11:J12" si="11">D11*$J$3</f>
         <v>0</v>
       </c>
       <c r="K11" s="12">
-        <f t="shared" si="9"/>
+        <f t="shared" ref="K11:K12" si="12">E11*$K$3</f>
         <v>99300</v>
       </c>
       <c r="L11" s="12">
-        <f t="shared" si="10"/>
+        <f t="shared" ref="L11:L12" si="13">F11*$L$3</f>
         <v>0</v>
       </c>
       <c r="M11" s="12">
-        <f t="shared" si="1"/>
+        <f t="shared" ref="M11:M12" si="14">G11*$M$3</f>
         <v>0</v>
       </c>
       <c r="N11" s="12">
-        <f t="shared" si="2"/>
+        <f t="shared" ref="N11:N12" si="15">H11*$N$3</f>
         <v>0</v>
       </c>
       <c r="O11" s="12">
-        <f t="shared" si="3"/>
+        <f t="shared" ref="O11:O12" si="16">SUM(J11:N11)</f>
         <v>99300</v>
       </c>
       <c r="P11" s="12">
-        <f t="shared" si="4"/>
+        <f t="shared" ref="P11:P12" si="17">I11*30%</f>
         <v>99300</v>
       </c>
       <c r="Q11" s="12">
-        <f t="shared" si="5"/>
+        <f t="shared" ref="Q11:Q12" si="18">O11-P11</f>
         <v>0</v>
       </c>
       <c r="R11" s="13">
@@ -2036,20 +2036,20 @@
       <c r="Z11" s="14"/>
       <c r="AA11" s="14"/>
       <c r="AB11" s="12">
-        <f t="shared" si="6"/>
+        <f t="shared" ref="AB11:AB12" si="19">SUM(S11:AA11)</f>
         <v>52500</v>
       </c>
       <c r="AC11" s="12">
         <v>0</v>
       </c>
       <c r="AD11" s="12">
-        <f t="shared" si="7"/>
+        <f t="shared" ref="AD11:AD12" si="20">O11-AB11</f>
         <v>46800</v>
       </c>
       <c r="AE11" s="14"/>
       <c r="AF11" s="14"/>
       <c r="AG11" s="12">
-        <f t="shared" si="8"/>
+        <f t="shared" ref="AG11:AG12" si="21">AE11+AF11</f>
         <v>0</v>
       </c>
     </row>
@@ -2082,35 +2082,35 @@
         <v>150000</v>
       </c>
       <c r="J12" s="12">
-        <f t="shared" si="0"/>
+        <f t="shared" si="11"/>
         <v>30000</v>
       </c>
       <c r="K12" s="12">
-        <f t="shared" si="9"/>
+        <f t="shared" si="12"/>
         <v>0</v>
       </c>
       <c r="L12" s="12">
-        <f t="shared" si="10"/>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
       <c r="M12" s="12">
-        <f t="shared" si="1"/>
+        <f t="shared" si="14"/>
         <v>0</v>
       </c>
       <c r="N12" s="12">
-        <f t="shared" si="2"/>
+        <f t="shared" si="15"/>
         <v>0</v>
       </c>
       <c r="O12" s="12">
-        <f t="shared" si="3"/>
+        <f t="shared" si="16"/>
         <v>30000</v>
       </c>
       <c r="P12" s="12">
-        <f t="shared" si="4"/>
+        <f t="shared" si="17"/>
         <v>45000</v>
       </c>
       <c r="Q12" s="12">
-        <f t="shared" si="5"/>
+        <f t="shared" si="18"/>
         <v>-15000</v>
       </c>
       <c r="R12" s="13">
@@ -2126,222 +2126,335 @@
       <c r="Z12" s="14"/>
       <c r="AA12" s="14"/>
       <c r="AB12" s="12">
-        <f t="shared" si="6"/>
+        <f t="shared" si="19"/>
         <v>0</v>
       </c>
       <c r="AC12" s="12">
         <v>0</v>
       </c>
       <c r="AD12" s="12">
-        <f t="shared" si="7"/>
+        <f t="shared" si="20"/>
         <v>30000</v>
       </c>
       <c r="AE12" s="14"/>
       <c r="AF12" s="14"/>
       <c r="AG12" s="12">
+        <f t="shared" si="21"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:33">
+      <c r="A13" s="11" t="s">
+        <v>4</v>
+      </c>
+      <c r="B13" s="11" t="s">
+        <v>42</v>
+      </c>
+      <c r="C13" s="12">
+        <v>1</v>
+      </c>
+      <c r="D13" s="12">
+        <v>0</v>
+      </c>
+      <c r="E13" s="12">
+        <v>331000</v>
+      </c>
+      <c r="F13" s="12">
+        <v>0</v>
+      </c>
+      <c r="G13" s="12">
+        <v>0</v>
+      </c>
+      <c r="H13" s="12">
+        <v>0</v>
+      </c>
+      <c r="I13" s="12">
+        <v>331000</v>
+      </c>
+      <c r="J13" s="12">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="K13" s="12">
+        <f t="shared" si="9"/>
+        <v>99300</v>
+      </c>
+      <c r="L13" s="12">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
+      <c r="M13" s="12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="N13" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="O13" s="12">
+        <f t="shared" si="3"/>
+        <v>99300</v>
+      </c>
+      <c r="P13" s="12">
+        <f t="shared" si="4"/>
+        <v>99300</v>
+      </c>
+      <c r="Q13" s="12">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="R13" s="13">
+        <v>30</v>
+      </c>
+      <c r="S13" s="14">
+        <f>175000*30%</f>
+        <v>52500</v>
+      </c>
+      <c r="T13" s="14"/>
+      <c r="U13" s="14"/>
+      <c r="V13" s="14"/>
+      <c r="W13" s="14"/>
+      <c r="X13" s="14"/>
+      <c r="Y13" s="14"/>
+      <c r="Z13" s="14"/>
+      <c r="AA13" s="14"/>
+      <c r="AB13" s="12">
+        <f t="shared" si="6"/>
+        <v>52500</v>
+      </c>
+      <c r="AC13" s="12">
+        <v>0</v>
+      </c>
+      <c r="AD13" s="12">
+        <f t="shared" si="7"/>
+        <v>46800</v>
+      </c>
+      <c r="AE13" s="14"/>
+      <c r="AF13" s="14"/>
+      <c r="AG13" s="12">
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:33">
-      <c r="A13" s="19" t="s">
+    <row r="14" spans="1:33">
+      <c r="A14" s="11" t="s">
+        <v>45</v>
+      </c>
+      <c r="B14" s="11" t="s">
+        <v>42</v>
+      </c>
+      <c r="C14" s="12">
+        <v>1</v>
+      </c>
+      <c r="D14" s="12">
+        <v>150000</v>
+      </c>
+      <c r="E14" s="12">
+        <v>0</v>
+      </c>
+      <c r="F14" s="12">
+        <v>0</v>
+      </c>
+      <c r="G14" s="12">
+        <v>0</v>
+      </c>
+      <c r="H14" s="12">
+        <v>0</v>
+      </c>
+      <c r="I14" s="12">
+        <v>150000</v>
+      </c>
+      <c r="J14" s="12">
+        <f t="shared" si="0"/>
+        <v>30000</v>
+      </c>
+      <c r="K14" s="12">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="L14" s="12">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
+      <c r="M14" s="12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="N14" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="O14" s="12">
+        <f t="shared" si="3"/>
+        <v>30000</v>
+      </c>
+      <c r="P14" s="12">
+        <f t="shared" si="4"/>
+        <v>45000</v>
+      </c>
+      <c r="Q14" s="12">
+        <f t="shared" si="5"/>
+        <v>-15000</v>
+      </c>
+      <c r="R14" s="13">
+        <v>20</v>
+      </c>
+      <c r="S14" s="14"/>
+      <c r="T14" s="14"/>
+      <c r="U14" s="14"/>
+      <c r="V14" s="14"/>
+      <c r="W14" s="14"/>
+      <c r="X14" s="14"/>
+      <c r="Y14" s="14"/>
+      <c r="Z14" s="14"/>
+      <c r="AA14" s="14"/>
+      <c r="AB14" s="12">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="AC14" s="12">
+        <v>0</v>
+      </c>
+      <c r="AD14" s="12">
+        <f t="shared" si="7"/>
+        <v>30000</v>
+      </c>
+      <c r="AE14" s="14"/>
+      <c r="AF14" s="14"/>
+      <c r="AG14" s="12">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:33">
+      <c r="A15" s="19" t="s">
         <v>46</v>
       </c>
-      <c r="B13" s="19"/>
-      <c r="C13" s="20">
-        <f t="shared" ref="C13:Q13" si="11">SUM(C5:C12)</f>
-        <v>582</v>
-      </c>
-      <c r="D13" s="20">
-        <f t="shared" si="11"/>
-        <v>73279250</v>
-      </c>
-      <c r="E13" s="20">
-        <f t="shared" si="11"/>
-        <v>62516500</v>
-      </c>
-      <c r="F13" s="20">
-        <f t="shared" si="11"/>
+      <c r="B15" s="19"/>
+      <c r="C15" s="20">
+        <f>SUM(C5:C14)</f>
+        <v>584</v>
+      </c>
+      <c r="D15" s="20">
+        <f>SUM(D5:D14)</f>
+        <v>73429250</v>
+      </c>
+      <c r="E15" s="20">
+        <f>SUM(E5:E14)</f>
+        <v>62847500</v>
+      </c>
+      <c r="F15" s="20">
+        <f>SUM(F5:F14)</f>
         <v>20319000</v>
       </c>
-      <c r="G13" s="20">
-        <f t="shared" si="11"/>
-        <v>0</v>
-      </c>
-      <c r="H13" s="20">
-        <f t="shared" si="11"/>
+      <c r="G15" s="20">
+        <f>SUM(G5:G14)</f>
+        <v>0</v>
+      </c>
+      <c r="H15" s="20">
+        <f>SUM(H5:H14)</f>
         <v>9458000</v>
       </c>
-      <c r="I13" s="20">
-        <f t="shared" si="11"/>
-        <v>165572750</v>
-      </c>
-      <c r="J13" s="20">
-        <f t="shared" si="11"/>
-        <v>14655850</v>
-      </c>
-      <c r="K13" s="20">
-        <f t="shared" si="11"/>
-        <v>19356595</v>
-      </c>
-      <c r="L13" s="20">
-        <f t="shared" si="11"/>
+      <c r="I15" s="20">
+        <f>SUM(I5:I14)</f>
+        <v>166053750</v>
+      </c>
+      <c r="J15" s="20">
+        <f>SUM(J5:J14)</f>
+        <v>14685850</v>
+      </c>
+      <c r="K15" s="20">
+        <f>SUM(K5:K14)</f>
+        <v>19455895</v>
+      </c>
+      <c r="L15" s="20">
+        <f>SUM(L5:L14)</f>
         <v>6802875</v>
       </c>
-      <c r="M13" s="20">
-        <f t="shared" si="11"/>
-        <v>0</v>
-      </c>
-      <c r="N13" s="20">
-        <f t="shared" si="11"/>
+      <c r="M15" s="20">
+        <f>SUM(M5:M14)</f>
+        <v>0</v>
+      </c>
+      <c r="N15" s="20">
+        <f>SUM(N5:N14)</f>
         <v>2837400</v>
       </c>
-      <c r="O13" s="20">
-        <f t="shared" si="11"/>
-        <v>43652720</v>
-      </c>
-      <c r="P13" s="20">
-        <f t="shared" si="11"/>
-        <v>49671825</v>
-      </c>
-      <c r="Q13" s="20">
-        <f t="shared" si="11"/>
-        <v>-6019105</v>
-      </c>
-      <c r="R13" s="21">
-        <f>IF(I13=0,0,O13/I13*100)</f>
-        <v>26.364676554565889</v>
-      </c>
-      <c r="S13" s="20">
-        <f t="shared" ref="S13:AG13" si="12">SUM(S5:S12)</f>
-        <v>343800</v>
-      </c>
-      <c r="T13" s="20">
-        <f t="shared" si="12"/>
-        <v>0</v>
-      </c>
-      <c r="U13" s="20">
-        <f t="shared" si="12"/>
+      <c r="O15" s="20">
+        <f>SUM(O5:O14)</f>
+        <v>43782020</v>
+      </c>
+      <c r="P15" s="20">
+        <f>SUM(P5:P14)</f>
+        <v>49816125</v>
+      </c>
+      <c r="Q15" s="20">
+        <f>SUM(Q5:Q14)</f>
+        <v>-6034105</v>
+      </c>
+      <c r="R15" s="21">
+        <f>IF(I15=0,0,O15/I15*100)</f>
+        <v>26.366173603426603</v>
+      </c>
+      <c r="S15" s="20">
+        <f t="shared" ref="S15:AG15" si="22">SUM(S5:S14)</f>
+        <v>396300</v>
+      </c>
+      <c r="T15" s="20">
+        <f t="shared" si="22"/>
+        <v>0</v>
+      </c>
+      <c r="U15" s="20">
+        <f t="shared" si="22"/>
         <v>343805</v>
       </c>
-      <c r="V13" s="20">
-        <f t="shared" si="12"/>
-        <v>0</v>
-      </c>
-      <c r="W13" s="20">
-        <f t="shared" si="12"/>
-        <v>0</v>
-      </c>
-      <c r="X13" s="20">
-        <f t="shared" si="12"/>
-        <v>0</v>
-      </c>
-      <c r="Y13" s="20">
-        <f t="shared" si="12"/>
+      <c r="V15" s="20">
+        <f t="shared" si="22"/>
+        <v>0</v>
+      </c>
+      <c r="W15" s="20">
+        <f t="shared" si="22"/>
+        <v>0</v>
+      </c>
+      <c r="X15" s="20">
+        <f t="shared" si="22"/>
+        <v>0</v>
+      </c>
+      <c r="Y15" s="20">
+        <f t="shared" si="22"/>
         <v>30000</v>
       </c>
-      <c r="Z13" s="20">
-        <f t="shared" si="12"/>
+      <c r="Z15" s="20">
+        <f t="shared" si="22"/>
         <v>100000</v>
       </c>
-      <c r="AA13" s="20">
-        <f t="shared" si="12"/>
+      <c r="AA15" s="20">
+        <f t="shared" si="22"/>
         <v>500000</v>
       </c>
-      <c r="AB13" s="20">
-        <f t="shared" si="12"/>
-        <v>1317605</v>
-      </c>
-      <c r="AC13" s="20">
-        <f t="shared" si="12"/>
-        <v>0</v>
-      </c>
-      <c r="AD13" s="20">
-        <f t="shared" si="12"/>
-        <v>42335115</v>
-      </c>
-      <c r="AE13" s="20">
-        <f t="shared" si="12"/>
+      <c r="AB15" s="20">
+        <f t="shared" si="22"/>
+        <v>1370105</v>
+      </c>
+      <c r="AC15" s="20">
+        <f t="shared" si="22"/>
+        <v>0</v>
+      </c>
+      <c r="AD15" s="20">
+        <f t="shared" si="22"/>
+        <v>42411915</v>
+      </c>
+      <c r="AE15" s="20">
+        <f t="shared" si="22"/>
         <v>1165600</v>
       </c>
-      <c r="AF13" s="20">
-        <f t="shared" si="12"/>
+      <c r="AF15" s="20">
+        <f t="shared" si="22"/>
         <v>51560605.149999999</v>
       </c>
-      <c r="AG13" s="20">
-        <f t="shared" si="12"/>
+      <c r="AG15" s="20">
+        <f t="shared" si="22"/>
         <v>52726205.149999999</v>
       </c>
-    </row>
-    <row r="14" spans="1:33">
-      <c r="A14" s="2"/>
-      <c r="B14" s="2"/>
-      <c r="C14" s="2"/>
-      <c r="D14" s="2"/>
-      <c r="E14" s="2"/>
-      <c r="F14" s="2"/>
-      <c r="G14" s="2"/>
-      <c r="H14" s="2"/>
-      <c r="I14" s="2"/>
-      <c r="J14" s="2"/>
-      <c r="K14" s="2"/>
-      <c r="L14" s="2"/>
-      <c r="M14" s="2"/>
-      <c r="N14" s="2"/>
-      <c r="O14" s="2"/>
-      <c r="P14" s="2"/>
-      <c r="Q14" s="2"/>
-      <c r="R14" s="2"/>
-      <c r="S14" s="2"/>
-      <c r="T14" s="2"/>
-      <c r="U14" s="2"/>
-      <c r="V14" s="2"/>
-      <c r="W14" s="2"/>
-      <c r="X14" s="2"/>
-      <c r="Y14" s="2"/>
-      <c r="Z14" s="2"/>
-      <c r="AA14" s="2"/>
-      <c r="AB14" s="2"/>
-      <c r="AC14" s="2"/>
-      <c r="AD14" s="2"/>
-      <c r="AE14" s="2"/>
-      <c r="AF14" s="2"/>
-      <c r="AG14" s="2"/>
-    </row>
-    <row r="15" spans="1:33">
-      <c r="A15" s="2"/>
-      <c r="B15" s="2"/>
-      <c r="C15" s="2"/>
-      <c r="D15" s="2"/>
-      <c r="E15" s="2"/>
-      <c r="F15" s="2"/>
-      <c r="G15" s="2"/>
-      <c r="H15" s="2"/>
-      <c r="I15" s="2"/>
-      <c r="J15" s="2"/>
-      <c r="K15" s="2"/>
-      <c r="L15" s="2"/>
-      <c r="M15" s="2"/>
-      <c r="N15" s="2"/>
-      <c r="O15" s="2"/>
-      <c r="P15" s="2"/>
-      <c r="Q15" s="2"/>
-      <c r="R15" s="2"/>
-      <c r="S15" s="2"/>
-      <c r="T15" s="2"/>
-      <c r="U15" s="2"/>
-      <c r="V15" s="2"/>
-      <c r="W15" s="2"/>
-      <c r="X15" s="2"/>
-      <c r="Y15" s="2"/>
-      <c r="Z15" s="2"/>
-      <c r="AA15" s="2"/>
-      <c r="AB15" s="2"/>
-      <c r="AC15" s="2"/>
-      <c r="AD15" s="2"/>
-      <c r="AE15" s="2"/>
-      <c r="AF15" s="2"/>
-      <c r="AG15" s="2"/>
     </row>
     <row r="16" spans="1:33">
       <c r="A16" s="2"/>
@@ -2518,7 +2631,7 @@
       <c r="AF20" s="2"/>
       <c r="AG20" s="2"/>
     </row>
-    <row r="21" spans="1:33" ht="15.75" customHeight="1">
+    <row r="21" spans="1:33">
       <c r="A21" s="2"/>
       <c r="B21" s="2"/>
       <c r="C21" s="2"/>
@@ -2553,7 +2666,7 @@
       <c r="AF21" s="2"/>
       <c r="AG21" s="2"/>
     </row>
-    <row r="22" spans="1:33" ht="15.75" customHeight="1">
+    <row r="22" spans="1:33">
       <c r="A22" s="2"/>
       <c r="B22" s="2"/>
       <c r="C22" s="2"/>
@@ -5318,6 +5431,76 @@
       <c r="AF100" s="2"/>
       <c r="AG100" s="2"/>
     </row>
+    <row r="101" spans="1:33" ht="15.75" customHeight="1">
+      <c r="A101" s="2"/>
+      <c r="B101" s="2"/>
+      <c r="C101" s="2"/>
+      <c r="D101" s="2"/>
+      <c r="E101" s="2"/>
+      <c r="F101" s="2"/>
+      <c r="G101" s="2"/>
+      <c r="H101" s="2"/>
+      <c r="I101" s="2"/>
+      <c r="J101" s="2"/>
+      <c r="K101" s="2"/>
+      <c r="L101" s="2"/>
+      <c r="M101" s="2"/>
+      <c r="N101" s="2"/>
+      <c r="O101" s="2"/>
+      <c r="P101" s="2"/>
+      <c r="Q101" s="2"/>
+      <c r="R101" s="2"/>
+      <c r="S101" s="2"/>
+      <c r="T101" s="2"/>
+      <c r="U101" s="2"/>
+      <c r="V101" s="2"/>
+      <c r="W101" s="2"/>
+      <c r="X101" s="2"/>
+      <c r="Y101" s="2"/>
+      <c r="Z101" s="2"/>
+      <c r="AA101" s="2"/>
+      <c r="AB101" s="2"/>
+      <c r="AC101" s="2"/>
+      <c r="AD101" s="2"/>
+      <c r="AE101" s="2"/>
+      <c r="AF101" s="2"/>
+      <c r="AG101" s="2"/>
+    </row>
+    <row r="102" spans="1:33" ht="15.75" customHeight="1">
+      <c r="A102" s="2"/>
+      <c r="B102" s="2"/>
+      <c r="C102" s="2"/>
+      <c r="D102" s="2"/>
+      <c r="E102" s="2"/>
+      <c r="F102" s="2"/>
+      <c r="G102" s="2"/>
+      <c r="H102" s="2"/>
+      <c r="I102" s="2"/>
+      <c r="J102" s="2"/>
+      <c r="K102" s="2"/>
+      <c r="L102" s="2"/>
+      <c r="M102" s="2"/>
+      <c r="N102" s="2"/>
+      <c r="O102" s="2"/>
+      <c r="P102" s="2"/>
+      <c r="Q102" s="2"/>
+      <c r="R102" s="2"/>
+      <c r="S102" s="2"/>
+      <c r="T102" s="2"/>
+      <c r="U102" s="2"/>
+      <c r="V102" s="2"/>
+      <c r="W102" s="2"/>
+      <c r="X102" s="2"/>
+      <c r="Y102" s="2"/>
+      <c r="Z102" s="2"/>
+      <c r="AA102" s="2"/>
+      <c r="AB102" s="2"/>
+      <c r="AC102" s="2"/>
+      <c r="AD102" s="2"/>
+      <c r="AE102" s="2"/>
+      <c r="AF102" s="2"/>
+      <c r="AG102" s="2"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0" footer="0"/>
   <pageSetup orientation="landscape"/>
@@ -5329,7 +5512,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AH100"/>
+  <dimension ref="A1:AH102"/>
   <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="1.42578125" customWidth="1"/>
@@ -5690,7 +5873,7 @@
       <c r="H8" s="42"/>
       <c r="I8" s="45"/>
       <c r="J8" s="42" t="str">
-        <f t="shared" ref="J8:J15" si="0">CONCATENATE($G$7,G8,$H$7,H8,$I$7,I8)</f>
+        <f t="shared" ref="J8:J17" si="0">CONCATENATE($G$7,G8,$H$7,H8,$I$7,I8)</f>
         <v xml:space="preserve">Bank BSI No. Rek.  A/n </v>
       </c>
       <c r="K8" s="42" t="s">
@@ -5709,7 +5892,7 @@
         <v>0</v>
       </c>
       <c r="O8" s="47">
-        <f t="shared" ref="O8:O15" si="1">SUM(M8:N8)</f>
+        <f t="shared" ref="O8:O17" si="1">SUM(M8:N8)</f>
         <v>10714040</v>
       </c>
       <c r="P8" s="47">
@@ -5753,11 +5936,11 @@
         <v>100000</v>
       </c>
       <c r="Z8" s="47">
-        <f t="shared" ref="Z8:Z15" si="2">O8-Y8</f>
+        <f t="shared" ref="Z8:Z17" si="2">O8-Y8</f>
         <v>10614040</v>
       </c>
       <c r="AA8" s="48" t="e">
-        <f t="shared" ref="AA8:AA15" ca="1" si="3">_xludf.TEXTJOIN(" | ",TRUE,IF(V8&gt;0,"Biaya Pendaftaran Koperasi: "&amp;TEXT(V8,"#.##0"),""),IF(W8&gt;0,"Simpanan Pokok: "&amp;TEXT(W8,"#.##0"),""),IF(X8&gt;0,"Simpanan Wajib: "&amp;TEXT(X8,"#.##0"),""))</f>
+        <f t="shared" ref="AA8:AA17" ca="1" si="3">_xludf.TEXTJOIN(" | ",TRUE,IF(V8&gt;0,"Biaya Pendaftaran Koperasi: "&amp;TEXT(V8,"#.##0"),""),IF(W8&gt;0,"Simpanan Pokok: "&amp;TEXT(W8,"#.##0"),""),IF(X8&gt;0,"Simpanan Wajib: "&amp;TEXT(X8,"#.##0"),""))</f>
         <v>#NAME?</v>
       </c>
       <c r="AB8" s="41"/>
@@ -5810,7 +5993,7 @@
         <v>0</v>
       </c>
       <c r="O9" s="47">
-        <f t="shared" si="1"/>
+        <f t="shared" ref="O9:O17" si="4">SUM(M9:N9)</f>
         <v>10252520</v>
       </c>
       <c r="P9" s="47">
@@ -5854,11 +6037,11 @@
         <v>443805</v>
       </c>
       <c r="Z9" s="47">
-        <f t="shared" si="2"/>
+        <f t="shared" ref="Z9:Z17" si="5">O9-Y9</f>
         <v>9808715</v>
       </c>
       <c r="AA9" s="48" t="e">
-        <f t="shared" ca="1" si="3"/>
+        <f t="shared" ref="AA9:AA17" ca="1" si="6">_xludf.TEXTJOIN(" | ",TRUE,IF(V9&gt;0,"Biaya Pendaftaran Koperasi: "&amp;TEXT(V9,"#.##0"),""),IF(W9&gt;0,"Simpanan Pokok: "&amp;TEXT(W9,"#.##0"),""),IF(X9&gt;0,"Simpanan Wajib: "&amp;TEXT(X9,"#.##0"),""))</f>
         <v>#NAME?</v>
       </c>
       <c r="AB9" s="41"/>
@@ -5911,7 +6094,7 @@
         <v>0</v>
       </c>
       <c r="O10" s="47">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>8265240</v>
       </c>
       <c r="P10" s="47">
@@ -5955,11 +6138,11 @@
         <v>184300</v>
       </c>
       <c r="Z10" s="47">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>8080940</v>
       </c>
       <c r="AA10" s="48" t="e">
-        <f t="shared" ca="1" si="3"/>
+        <f t="shared" ca="1" si="6"/>
         <v>#NAME?</v>
       </c>
       <c r="AB10" s="41"/>
@@ -6012,7 +6195,7 @@
         <v>0</v>
       </c>
       <c r="O11" s="47">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>5870920</v>
       </c>
       <c r="P11" s="47">
@@ -6056,11 +6239,11 @@
         <v>160000</v>
       </c>
       <c r="Z11" s="47">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>5710920</v>
       </c>
       <c r="AA11" s="48" t="e">
-        <f t="shared" ca="1" si="3"/>
+        <f t="shared" ca="1" si="6"/>
         <v>#NAME?</v>
       </c>
       <c r="AB11" s="41"/>
@@ -6113,7 +6296,7 @@
         <v>0</v>
       </c>
       <c r="O12" s="47">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>4266200</v>
       </c>
       <c r="P12" s="47">
@@ -6157,11 +6340,11 @@
         <v>157000</v>
       </c>
       <c r="Z12" s="47">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>4109200</v>
       </c>
       <c r="AA12" s="48" t="e">
-        <f t="shared" ca="1" si="3"/>
+        <f t="shared" ca="1" si="6"/>
         <v>#NAME?</v>
       </c>
       <c r="AB12" s="41"/>
@@ -6214,7 +6397,7 @@
         <v>0</v>
       </c>
       <c r="O13" s="47">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>4154500</v>
       </c>
       <c r="P13" s="47">
@@ -6258,11 +6441,11 @@
         <v>220000</v>
       </c>
       <c r="Z13" s="47">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>3934500</v>
       </c>
       <c r="AA13" s="48" t="e">
-        <f t="shared" ca="1" si="3"/>
+        <f t="shared" ca="1" si="6"/>
         <v>#NAME?</v>
       </c>
       <c r="AB13" s="41"/>
@@ -6315,7 +6498,7 @@
         <v>0</v>
       </c>
       <c r="O14" s="47">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>99300</v>
       </c>
       <c r="P14" s="47">
@@ -6359,11 +6542,11 @@
         <v>52500</v>
       </c>
       <c r="Z14" s="47">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>46800</v>
       </c>
       <c r="AA14" s="48" t="e">
-        <f t="shared" ca="1" si="3"/>
+        <f t="shared" ca="1" si="6"/>
         <v>#NAME?</v>
       </c>
       <c r="AB14" s="41"/>
@@ -6397,7 +6580,7 @@
       <c r="H15" s="42"/>
       <c r="I15" s="44"/>
       <c r="J15" s="42" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" ref="J15" si="7">CONCATENATE($G$7,G15,$H$7,H15,$I$7,I15)</f>
         <v xml:space="preserve">Bank BSI No. Rek.  A/n </v>
       </c>
       <c r="K15" s="42" t="s">
@@ -6416,7 +6599,7 @@
         <v>0</v>
       </c>
       <c r="O15" s="47">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>30000</v>
       </c>
       <c r="P15" s="47">
@@ -6460,11 +6643,11 @@
         <v>0</v>
       </c>
       <c r="Z15" s="47">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>30000</v>
       </c>
       <c r="AA15" s="48" t="e">
-        <f t="shared" ca="1" si="3"/>
+        <f t="shared" ca="1" si="6"/>
         <v>#NAME?</v>
       </c>
       <c r="AB15" s="41"/>
@@ -6475,194 +6658,319 @@
       <c r="AG15" s="41"/>
       <c r="AH15" s="41"/>
     </row>
-    <row r="16" spans="1:34" ht="69" customHeight="1">
-      <c r="A16" s="49"/>
-      <c r="B16" s="65" t="s">
-        <v>46</v>
-      </c>
-      <c r="C16" s="66"/>
-      <c r="D16" s="66"/>
-      <c r="E16" s="66"/>
-      <c r="F16" s="66"/>
-      <c r="G16" s="66"/>
-      <c r="H16" s="66"/>
-      <c r="I16" s="66"/>
-      <c r="J16" s="66"/>
-      <c r="K16" s="67"/>
-      <c r="L16" s="50">
-        <f t="shared" ref="L16:Z16" si="4">SUM(L8:L15)</f>
-        <v>165572750</v>
-      </c>
-      <c r="M16" s="50">
+    <row r="16" spans="1:34" ht="60" customHeight="1">
+      <c r="A16" s="41"/>
+      <c r="B16" s="42">
+        <v>9</v>
+      </c>
+      <c r="C16" s="43"/>
+      <c r="D16" s="44" t="str">
+        <f>RAW!A13</f>
+        <v>YUVI NOFERIANTO</v>
+      </c>
+      <c r="E16" s="44" t="s">
+        <v>67</v>
+      </c>
+      <c r="F16" s="42" t="str">
+        <f>RAW!B13</f>
+        <v>JATIMULYA</v>
+      </c>
+      <c r="G16" s="42" t="s">
+        <v>68</v>
+      </c>
+      <c r="H16" s="42"/>
+      <c r="I16" s="44"/>
+      <c r="J16" s="42" t="str">
+        <f t="shared" ref="J16" si="8">CONCATENATE($G$7,G16,$H$7,H16,$I$7,I16)</f>
+        <v xml:space="preserve">Bank BSI No. Rek.  A/n </v>
+      </c>
+      <c r="K16" s="42" t="s">
+        <v>69</v>
+      </c>
+      <c r="L16" s="46">
+        <f>RAW!I13</f>
+        <v>331000</v>
+      </c>
+      <c r="M16" s="46">
+        <f>RAW!O13</f>
+        <v>99300</v>
+      </c>
+      <c r="N16" s="47">
+        <f>RAW!AC13</f>
+        <v>0</v>
+      </c>
+      <c r="O16" s="47">
         <f t="shared" si="4"/>
-        <v>43652720</v>
-      </c>
-      <c r="N16" s="50">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="O16" s="50">
-        <f t="shared" si="4"/>
-        <v>43652720</v>
-      </c>
-      <c r="P16" s="50">
-        <f t="shared" si="4"/>
-        <v>343800</v>
-      </c>
-      <c r="Q16" s="50">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="R16" s="50">
-        <f t="shared" si="4"/>
-        <v>343805</v>
-      </c>
-      <c r="S16" s="50">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="T16" s="50">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="U16" s="50">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="V16" s="50">
+        <v>99300</v>
+      </c>
+      <c r="P16" s="47">
+        <f>RAW!S13</f>
+        <v>52500</v>
+      </c>
+      <c r="Q16" s="47">
+        <f>RAW!T13</f>
+        <v>0</v>
+      </c>
+      <c r="R16" s="47">
+        <f>RAW!U13</f>
+        <v>0</v>
+      </c>
+      <c r="S16" s="47">
+        <f>RAW!V13</f>
+        <v>0</v>
+      </c>
+      <c r="T16" s="47">
+        <f>RAW!W13</f>
+        <v>0</v>
+      </c>
+      <c r="U16" s="47">
+        <f>RAW!X13</f>
+        <v>0</v>
+      </c>
+      <c r="V16" s="47">
+        <f>RAW!Y13</f>
+        <v>0</v>
+      </c>
+      <c r="W16" s="47">
+        <f>RAW!Z13</f>
+        <v>0</v>
+      </c>
+      <c r="X16" s="47">
+        <f>RAW!AA13</f>
+        <v>0</v>
+      </c>
+      <c r="Y16" s="47">
+        <f>RAW!AB13</f>
+        <v>52500</v>
+      </c>
+      <c r="Z16" s="47">
+        <f t="shared" si="5"/>
+        <v>46800</v>
+      </c>
+      <c r="AA16" s="48" t="e">
+        <f t="shared" ca="1" si="6"/>
+        <v>#NAME?</v>
+      </c>
+      <c r="AB16" s="41"/>
+      <c r="AC16" s="41"/>
+      <c r="AD16" s="41"/>
+      <c r="AE16" s="41"/>
+      <c r="AF16" s="41"/>
+      <c r="AG16" s="41"/>
+      <c r="AH16" s="41"/>
+    </row>
+    <row r="17" spans="1:34" ht="60" customHeight="1">
+      <c r="A17" s="41"/>
+      <c r="B17" s="42">
+        <v>10</v>
+      </c>
+      <c r="C17" s="43"/>
+      <c r="D17" s="44" t="str">
+        <f>RAW!A14</f>
+        <v>IKANG TAUFIK (OPIK)</v>
+      </c>
+      <c r="E17" s="44" t="s">
+        <v>67</v>
+      </c>
+      <c r="F17" s="42" t="str">
+        <f>RAW!B14</f>
+        <v>JATIMULYA</v>
+      </c>
+      <c r="G17" s="42" t="s">
+        <v>68</v>
+      </c>
+      <c r="H17" s="42"/>
+      <c r="I17" s="44"/>
+      <c r="J17" s="42" t="str">
+        <f t="shared" si="0"/>
+        <v xml:space="preserve">Bank BSI No. Rek.  A/n </v>
+      </c>
+      <c r="K17" s="42" t="s">
+        <v>69</v>
+      </c>
+      <c r="L17" s="46">
+        <f>RAW!I14</f>
+        <v>150000</v>
+      </c>
+      <c r="M17" s="46">
+        <f>RAW!O14</f>
+        <v>30000</v>
+      </c>
+      <c r="N17" s="47">
+        <f>RAW!AC14</f>
+        <v>0</v>
+      </c>
+      <c r="O17" s="47">
         <f t="shared" si="4"/>
         <v>30000</v>
       </c>
-      <c r="W16" s="50">
-        <f t="shared" si="4"/>
+      <c r="P17" s="47">
+        <f>RAW!S14</f>
+        <v>0</v>
+      </c>
+      <c r="Q17" s="47">
+        <f>RAW!T14</f>
+        <v>0</v>
+      </c>
+      <c r="R17" s="47">
+        <f>RAW!U14</f>
+        <v>0</v>
+      </c>
+      <c r="S17" s="47">
+        <f>RAW!V14</f>
+        <v>0</v>
+      </c>
+      <c r="T17" s="47">
+        <f>RAW!W14</f>
+        <v>0</v>
+      </c>
+      <c r="U17" s="47">
+        <f>RAW!X14</f>
+        <v>0</v>
+      </c>
+      <c r="V17" s="47">
+        <f>RAW!Y14</f>
+        <v>0</v>
+      </c>
+      <c r="W17" s="47">
+        <f>RAW!Z14</f>
+        <v>0</v>
+      </c>
+      <c r="X17" s="47">
+        <f>RAW!AA14</f>
+        <v>0</v>
+      </c>
+      <c r="Y17" s="47">
+        <f>RAW!AB14</f>
+        <v>0</v>
+      </c>
+      <c r="Z17" s="47">
+        <f t="shared" si="5"/>
+        <v>30000</v>
+      </c>
+      <c r="AA17" s="48" t="e">
+        <f t="shared" ca="1" si="6"/>
+        <v>#NAME?</v>
+      </c>
+      <c r="AB17" s="41"/>
+      <c r="AC17" s="41"/>
+      <c r="AD17" s="41"/>
+      <c r="AE17" s="41"/>
+      <c r="AF17" s="41"/>
+      <c r="AG17" s="41"/>
+      <c r="AH17" s="41"/>
+    </row>
+    <row r="18" spans="1:34" ht="69" customHeight="1">
+      <c r="A18" s="49"/>
+      <c r="B18" s="65" t="s">
+        <v>46</v>
+      </c>
+      <c r="C18" s="66"/>
+      <c r="D18" s="66"/>
+      <c r="E18" s="66"/>
+      <c r="F18" s="66"/>
+      <c r="G18" s="66"/>
+      <c r="H18" s="66"/>
+      <c r="I18" s="66"/>
+      <c r="J18" s="66"/>
+      <c r="K18" s="67"/>
+      <c r="L18" s="50">
+        <f t="shared" ref="L18:Z18" si="9">SUM(L8:L17)</f>
+        <v>166053750</v>
+      </c>
+      <c r="M18" s="50">
+        <f t="shared" si="9"/>
+        <v>43782020</v>
+      </c>
+      <c r="N18" s="50">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="O18" s="50">
+        <f t="shared" si="9"/>
+        <v>43782020</v>
+      </c>
+      <c r="P18" s="50">
+        <f t="shared" si="9"/>
+        <v>396300</v>
+      </c>
+      <c r="Q18" s="50">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="R18" s="50">
+        <f t="shared" si="9"/>
+        <v>343805</v>
+      </c>
+      <c r="S18" s="50">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="T18" s="50">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="U18" s="50">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="V18" s="50">
+        <f t="shared" si="9"/>
+        <v>30000</v>
+      </c>
+      <c r="W18" s="50">
+        <f t="shared" si="9"/>
         <v>100000</v>
       </c>
-      <c r="X16" s="50">
-        <f t="shared" si="4"/>
+      <c r="X18" s="50">
+        <f t="shared" si="9"/>
         <v>500000</v>
       </c>
-      <c r="Y16" s="50">
-        <f t="shared" si="4"/>
-        <v>1317605</v>
-      </c>
-      <c r="Z16" s="50">
-        <f t="shared" si="4"/>
-        <v>42335115</v>
-      </c>
-      <c r="AA16" s="51"/>
-      <c r="AB16" s="49"/>
-      <c r="AC16" s="49"/>
-      <c r="AD16" s="49"/>
-      <c r="AE16" s="49"/>
-      <c r="AF16" s="49"/>
-      <c r="AG16" s="49"/>
-      <c r="AH16" s="49"/>
-    </row>
-    <row r="17" spans="1:34" ht="25.5" customHeight="1">
-      <c r="A17" s="22"/>
-      <c r="B17" s="31"/>
-      <c r="C17" s="30"/>
-      <c r="D17" s="31"/>
-      <c r="E17" s="31"/>
-      <c r="F17" s="31"/>
-      <c r="G17" s="31"/>
-      <c r="H17" s="31"/>
-      <c r="I17" s="31"/>
-      <c r="J17" s="31"/>
-      <c r="K17" s="31"/>
-      <c r="L17" s="31"/>
-      <c r="M17" s="31"/>
-      <c r="N17" s="31"/>
-      <c r="O17" s="31"/>
-      <c r="P17" s="31"/>
-      <c r="Q17" s="31"/>
-      <c r="R17" s="31"/>
-      <c r="S17" s="31"/>
-      <c r="T17" s="31"/>
-      <c r="U17" s="31"/>
-      <c r="V17" s="31"/>
-      <c r="W17" s="31"/>
-      <c r="X17" s="31"/>
-      <c r="Y17" s="31"/>
-      <c r="Z17" s="31"/>
-      <c r="AA17" s="52"/>
-      <c r="AB17" s="22"/>
-      <c r="AC17" s="22"/>
-      <c r="AD17" s="22"/>
-      <c r="AE17" s="22"/>
-      <c r="AF17" s="22"/>
-      <c r="AG17" s="22"/>
-      <c r="AH17" s="22"/>
-    </row>
-    <row r="18" spans="1:34" ht="14.25" customHeight="1">
-      <c r="A18" s="22"/>
-      <c r="B18" s="22"/>
-      <c r="C18" s="23"/>
-      <c r="D18" s="22"/>
-      <c r="E18" s="22"/>
-      <c r="F18" s="24"/>
-      <c r="G18" s="24"/>
-      <c r="H18" s="24"/>
-      <c r="I18" s="24"/>
-      <c r="J18" s="24"/>
-      <c r="K18" s="24"/>
-      <c r="L18" s="22"/>
-      <c r="M18" s="22"/>
-      <c r="N18" s="22"/>
-      <c r="O18" s="22"/>
-      <c r="P18" s="22"/>
-      <c r="Q18" s="22"/>
-      <c r="R18" s="22"/>
-      <c r="S18" s="22"/>
-      <c r="T18" s="22"/>
-      <c r="U18" s="22"/>
-      <c r="V18" s="22"/>
-      <c r="W18" s="22"/>
-      <c r="X18" s="22"/>
-      <c r="Y18" s="22"/>
-      <c r="Z18" s="22"/>
-      <c r="AA18" s="22"/>
-      <c r="AB18" s="22"/>
-      <c r="AC18" s="22"/>
-      <c r="AD18" s="22"/>
-      <c r="AE18" s="22"/>
-      <c r="AF18" s="22"/>
-      <c r="AG18" s="22"/>
-      <c r="AH18" s="22"/>
-    </row>
-    <row r="19" spans="1:34" ht="14.25" customHeight="1">
+      <c r="Y18" s="50">
+        <f t="shared" si="9"/>
+        <v>1370105</v>
+      </c>
+      <c r="Z18" s="50">
+        <f t="shared" si="9"/>
+        <v>42411915</v>
+      </c>
+      <c r="AA18" s="51"/>
+      <c r="AB18" s="49"/>
+      <c r="AC18" s="49"/>
+      <c r="AD18" s="49"/>
+      <c r="AE18" s="49"/>
+      <c r="AF18" s="49"/>
+      <c r="AG18" s="49"/>
+      <c r="AH18" s="49"/>
+    </row>
+    <row r="19" spans="1:34" ht="25.5" customHeight="1">
       <c r="A19" s="22"/>
-      <c r="B19" s="22"/>
-      <c r="C19" s="23"/>
-      <c r="D19" s="22"/>
-      <c r="E19" s="22"/>
-      <c r="F19" s="24"/>
-      <c r="G19" s="24"/>
-      <c r="H19" s="24"/>
-      <c r="I19" s="24"/>
-      <c r="J19" s="24"/>
-      <c r="K19" s="24"/>
-      <c r="L19" s="22"/>
-      <c r="M19" s="22"/>
-      <c r="N19" s="22"/>
-      <c r="O19" s="53" t="s">
-        <v>70</v>
-      </c>
-      <c r="P19" s="54">
-        <f ca="1">TODAY()</f>
-        <v>46262</v>
-      </c>
-      <c r="Q19" s="54"/>
-      <c r="R19" s="54"/>
-      <c r="S19" s="54"/>
-      <c r="T19" s="54"/>
-      <c r="U19" s="54"/>
-      <c r="V19" s="54"/>
-      <c r="W19" s="54"/>
-      <c r="X19" s="54"/>
-      <c r="Y19" s="22"/>
-      <c r="Z19" s="55"/>
-      <c r="AA19" s="22"/>
+      <c r="B19" s="31"/>
+      <c r="C19" s="30"/>
+      <c r="D19" s="31"/>
+      <c r="E19" s="31"/>
+      <c r="F19" s="31"/>
+      <c r="G19" s="31"/>
+      <c r="H19" s="31"/>
+      <c r="I19" s="31"/>
+      <c r="J19" s="31"/>
+      <c r="K19" s="31"/>
+      <c r="L19" s="31"/>
+      <c r="M19" s="31"/>
+      <c r="N19" s="31"/>
+      <c r="O19" s="31"/>
+      <c r="P19" s="31"/>
+      <c r="Q19" s="31"/>
+      <c r="R19" s="31"/>
+      <c r="S19" s="31"/>
+      <c r="T19" s="31"/>
+      <c r="U19" s="31"/>
+      <c r="V19" s="31"/>
+      <c r="W19" s="31"/>
+      <c r="X19" s="31"/>
+      <c r="Y19" s="31"/>
+      <c r="Z19" s="31"/>
+      <c r="AA19" s="52"/>
       <c r="AB19" s="22"/>
       <c r="AC19" s="22"/>
       <c r="AD19" s="22"/>
@@ -6671,117 +6979,122 @@
       <c r="AG19" s="22"/>
       <c r="AH19" s="22"/>
     </row>
-    <row r="20" spans="1:34" ht="57.75" customHeight="1">
-      <c r="A20" s="56"/>
-      <c r="B20" s="56"/>
-      <c r="C20" s="57"/>
-      <c r="D20" s="58" t="s">
-        <v>71</v>
-      </c>
-      <c r="E20" s="56"/>
-      <c r="F20" s="58"/>
-      <c r="G20" s="58"/>
-      <c r="H20" s="58"/>
-      <c r="I20" s="58"/>
-      <c r="J20" s="58"/>
-      <c r="K20" s="56"/>
-      <c r="L20" s="58"/>
-      <c r="M20" s="58"/>
-      <c r="N20" s="56"/>
-      <c r="O20" s="58" t="s">
-        <v>72</v>
-      </c>
-      <c r="P20" s="56"/>
-      <c r="Q20" s="56"/>
-      <c r="R20" s="56"/>
-      <c r="S20" s="58" t="s">
-        <v>72</v>
-      </c>
-      <c r="T20" s="58"/>
-      <c r="U20" s="58"/>
-      <c r="V20" s="58"/>
-      <c r="W20" s="58"/>
-      <c r="X20" s="58"/>
-      <c r="Y20" s="58" t="s">
-        <v>72</v>
-      </c>
-      <c r="Z20" s="59"/>
-      <c r="AA20" s="60"/>
-      <c r="AB20" s="56"/>
-      <c r="AC20" s="58"/>
-      <c r="AD20" s="58"/>
-      <c r="AE20" s="60"/>
-      <c r="AF20" s="60"/>
-      <c r="AG20" s="56"/>
-      <c r="AH20" s="56"/>
+    <row r="20" spans="1:34" ht="14.25" customHeight="1">
+      <c r="A20" s="22"/>
+      <c r="B20" s="22"/>
+      <c r="C20" s="23"/>
+      <c r="D20" s="22"/>
+      <c r="E20" s="22"/>
+      <c r="F20" s="24"/>
+      <c r="G20" s="24"/>
+      <c r="H20" s="24"/>
+      <c r="I20" s="24"/>
+      <c r="J20" s="24"/>
+      <c r="K20" s="24"/>
+      <c r="L20" s="22"/>
+      <c r="M20" s="22"/>
+      <c r="N20" s="22"/>
+      <c r="O20" s="22"/>
+      <c r="P20" s="22"/>
+      <c r="Q20" s="22"/>
+      <c r="R20" s="22"/>
+      <c r="S20" s="22"/>
+      <c r="T20" s="22"/>
+      <c r="U20" s="22"/>
+      <c r="V20" s="22"/>
+      <c r="W20" s="22"/>
+      <c r="X20" s="22"/>
+      <c r="Y20" s="22"/>
+      <c r="Z20" s="22"/>
+      <c r="AA20" s="22"/>
+      <c r="AB20" s="22"/>
+      <c r="AC20" s="22"/>
+      <c r="AD20" s="22"/>
+      <c r="AE20" s="22"/>
+      <c r="AF20" s="22"/>
+      <c r="AG20" s="22"/>
+      <c r="AH20" s="22"/>
     </row>
     <row r="21" spans="1:34" ht="14.25" customHeight="1">
-      <c r="A21" s="56"/>
-      <c r="B21" s="56"/>
-      <c r="C21" s="57"/>
-      <c r="D21" s="58"/>
-      <c r="E21" s="56"/>
-      <c r="F21" s="58"/>
-      <c r="G21" s="58"/>
-      <c r="H21" s="58"/>
-      <c r="I21" s="58"/>
-      <c r="J21" s="58"/>
-      <c r="K21" s="56"/>
-      <c r="L21" s="58"/>
-      <c r="M21" s="58"/>
-      <c r="N21" s="56"/>
-      <c r="O21" s="58"/>
-      <c r="P21" s="58"/>
-      <c r="Q21" s="58"/>
-      <c r="R21" s="58"/>
-      <c r="S21" s="58"/>
-      <c r="T21" s="58"/>
-      <c r="U21" s="58"/>
-      <c r="V21" s="58"/>
-      <c r="W21" s="58"/>
-      <c r="X21" s="58"/>
-      <c r="Y21" s="58"/>
-      <c r="Z21" s="59"/>
-      <c r="AA21" s="60"/>
-      <c r="AB21" s="58"/>
-      <c r="AC21" s="58"/>
-      <c r="AD21" s="58"/>
-      <c r="AE21" s="60"/>
-      <c r="AF21" s="60"/>
-      <c r="AG21" s="56"/>
-      <c r="AH21" s="56"/>
-    </row>
-    <row r="22" spans="1:34" ht="14.25" customHeight="1">
+      <c r="A21" s="22"/>
+      <c r="B21" s="22"/>
+      <c r="C21" s="23"/>
+      <c r="D21" s="22"/>
+      <c r="E21" s="22"/>
+      <c r="F21" s="24"/>
+      <c r="G21" s="24"/>
+      <c r="H21" s="24"/>
+      <c r="I21" s="24"/>
+      <c r="J21" s="24"/>
+      <c r="K21" s="24"/>
+      <c r="L21" s="22"/>
+      <c r="M21" s="22"/>
+      <c r="N21" s="22"/>
+      <c r="O21" s="53" t="s">
+        <v>70</v>
+      </c>
+      <c r="P21" s="54">
+        <f ca="1">TODAY()</f>
+        <v>46321</v>
+      </c>
+      <c r="Q21" s="54"/>
+      <c r="R21" s="54"/>
+      <c r="S21" s="54"/>
+      <c r="T21" s="54"/>
+      <c r="U21" s="54"/>
+      <c r="V21" s="54"/>
+      <c r="W21" s="54"/>
+      <c r="X21" s="54"/>
+      <c r="Y21" s="22"/>
+      <c r="Z21" s="55"/>
+      <c r="AA21" s="22"/>
+      <c r="AB21" s="22"/>
+      <c r="AC21" s="22"/>
+      <c r="AD21" s="22"/>
+      <c r="AE21" s="22"/>
+      <c r="AF21" s="22"/>
+      <c r="AG21" s="22"/>
+      <c r="AH21" s="22"/>
+    </row>
+    <row r="22" spans="1:34" ht="57.75" customHeight="1">
       <c r="A22" s="56"/>
       <c r="B22" s="56"/>
       <c r="C22" s="57"/>
-      <c r="D22" s="61"/>
+      <c r="D22" s="58" t="s">
+        <v>71</v>
+      </c>
       <c r="E22" s="56"/>
-      <c r="F22" s="56"/>
-      <c r="G22" s="56"/>
-      <c r="H22" s="56"/>
-      <c r="I22" s="56"/>
-      <c r="J22" s="56"/>
+      <c r="F22" s="58"/>
+      <c r="G22" s="58"/>
+      <c r="H22" s="58"/>
+      <c r="I22" s="58"/>
+      <c r="J22" s="58"/>
       <c r="K22" s="56"/>
-      <c r="L22" s="56"/>
-      <c r="M22" s="56"/>
+      <c r="L22" s="58"/>
+      <c r="M22" s="58"/>
       <c r="N22" s="56"/>
-      <c r="O22" s="56"/>
+      <c r="O22" s="58" t="s">
+        <v>72</v>
+      </c>
       <c r="P22" s="56"/>
       <c r="Q22" s="56"/>
       <c r="R22" s="56"/>
-      <c r="S22" s="56"/>
-      <c r="T22" s="56"/>
-      <c r="U22" s="56"/>
-      <c r="V22" s="56"/>
-      <c r="W22" s="56"/>
-      <c r="X22" s="56"/>
-      <c r="Y22" s="56"/>
-      <c r="Z22" s="62"/>
+      <c r="S22" s="58" t="s">
+        <v>72</v>
+      </c>
+      <c r="T22" s="58"/>
+      <c r="U22" s="58"/>
+      <c r="V22" s="58"/>
+      <c r="W22" s="58"/>
+      <c r="X22" s="58"/>
+      <c r="Y22" s="58" t="s">
+        <v>72</v>
+      </c>
+      <c r="Z22" s="59"/>
       <c r="AA22" s="60"/>
       <c r="AB22" s="56"/>
-      <c r="AC22" s="56"/>
-      <c r="AD22" s="56"/>
+      <c r="AC22" s="58"/>
+      <c r="AD22" s="58"/>
       <c r="AE22" s="60"/>
       <c r="AF22" s="60"/>
       <c r="AG22" s="56"/>
@@ -6791,33 +7104,33 @@
       <c r="A23" s="56"/>
       <c r="B23" s="56"/>
       <c r="C23" s="57"/>
-      <c r="D23" s="61"/>
+      <c r="D23" s="58"/>
       <c r="E23" s="56"/>
-      <c r="F23" s="56"/>
-      <c r="G23" s="56"/>
-      <c r="H23" s="56"/>
-      <c r="I23" s="56"/>
-      <c r="J23" s="56"/>
+      <c r="F23" s="58"/>
+      <c r="G23" s="58"/>
+      <c r="H23" s="58"/>
+      <c r="I23" s="58"/>
+      <c r="J23" s="58"/>
       <c r="K23" s="56"/>
-      <c r="L23" s="56"/>
-      <c r="M23" s="56"/>
+      <c r="L23" s="58"/>
+      <c r="M23" s="58"/>
       <c r="N23" s="56"/>
-      <c r="O23" s="56"/>
-      <c r="P23" s="63"/>
-      <c r="Q23" s="63"/>
-      <c r="R23" s="63"/>
-      <c r="S23" s="56"/>
-      <c r="T23" s="56"/>
-      <c r="U23" s="56"/>
-      <c r="V23" s="56"/>
-      <c r="W23" s="56"/>
-      <c r="X23" s="56"/>
-      <c r="Y23" s="56"/>
-      <c r="Z23" s="64"/>
+      <c r="O23" s="58"/>
+      <c r="P23" s="58"/>
+      <c r="Q23" s="58"/>
+      <c r="R23" s="58"/>
+      <c r="S23" s="58"/>
+      <c r="T23" s="58"/>
+      <c r="U23" s="58"/>
+      <c r="V23" s="58"/>
+      <c r="W23" s="58"/>
+      <c r="X23" s="58"/>
+      <c r="Y23" s="58"/>
+      <c r="Z23" s="59"/>
       <c r="AA23" s="60"/>
-      <c r="AB23" s="56"/>
-      <c r="AC23" s="56"/>
-      <c r="AD23" s="56"/>
+      <c r="AB23" s="58"/>
+      <c r="AC23" s="58"/>
+      <c r="AD23" s="58"/>
       <c r="AE23" s="60"/>
       <c r="AF23" s="60"/>
       <c r="AG23" s="56"/>
@@ -6849,7 +7162,7 @@
       <c r="W24" s="56"/>
       <c r="X24" s="56"/>
       <c r="Y24" s="56"/>
-      <c r="Z24" s="56"/>
+      <c r="Z24" s="62"/>
       <c r="AA24" s="60"/>
       <c r="AB24" s="56"/>
       <c r="AC24" s="56"/>
@@ -6863,7 +7176,7 @@
       <c r="A25" s="56"/>
       <c r="B25" s="56"/>
       <c r="C25" s="57"/>
-      <c r="D25" s="58"/>
+      <c r="D25" s="61"/>
       <c r="E25" s="56"/>
       <c r="F25" s="56"/>
       <c r="G25" s="56"/>
@@ -6875,9 +7188,9 @@
       <c r="M25" s="56"/>
       <c r="N25" s="56"/>
       <c r="O25" s="56"/>
-      <c r="P25" s="56"/>
-      <c r="Q25" s="56"/>
-      <c r="R25" s="56"/>
+      <c r="P25" s="63"/>
+      <c r="Q25" s="63"/>
+      <c r="R25" s="63"/>
       <c r="S25" s="56"/>
       <c r="T25" s="56"/>
       <c r="U25" s="56"/>
@@ -6886,12 +7199,12 @@
       <c r="X25" s="56"/>
       <c r="Y25" s="56"/>
       <c r="Z25" s="64"/>
-      <c r="AA25" s="56"/>
+      <c r="AA25" s="60"/>
       <c r="AB25" s="56"/>
       <c r="AC25" s="56"/>
       <c r="AD25" s="56"/>
-      <c r="AE25" s="56"/>
-      <c r="AF25" s="56"/>
+      <c r="AE25" s="60"/>
+      <c r="AF25" s="60"/>
       <c r="AG25" s="56"/>
       <c r="AH25" s="56"/>
     </row>
@@ -6899,7 +7212,7 @@
       <c r="A26" s="56"/>
       <c r="B26" s="56"/>
       <c r="C26" s="57"/>
-      <c r="D26" s="58"/>
+      <c r="D26" s="61"/>
       <c r="E26" s="56"/>
       <c r="F26" s="56"/>
       <c r="G26" s="56"/>
@@ -6921,23 +7234,21 @@
       <c r="W26" s="56"/>
       <c r="X26" s="56"/>
       <c r="Y26" s="56"/>
-      <c r="Z26" s="64"/>
-      <c r="AA26" s="56"/>
+      <c r="Z26" s="56"/>
+      <c r="AA26" s="60"/>
       <c r="AB26" s="56"/>
       <c r="AC26" s="56"/>
       <c r="AD26" s="56"/>
-      <c r="AE26" s="56"/>
-      <c r="AF26" s="56"/>
+      <c r="AE26" s="60"/>
+      <c r="AF26" s="60"/>
       <c r="AG26" s="56"/>
       <c r="AH26" s="56"/>
     </row>
-    <row r="27" spans="1:34" ht="33.75" customHeight="1">
+    <row r="27" spans="1:34" ht="14.25" customHeight="1">
       <c r="A27" s="56"/>
       <c r="B27" s="56"/>
       <c r="C27" s="57"/>
-      <c r="D27" s="58" t="s">
-        <v>73</v>
-      </c>
+      <c r="D27" s="58"/>
       <c r="E27" s="56"/>
       <c r="F27" s="56"/>
       <c r="G27" s="56"/>
@@ -6945,43 +7256,35 @@
       <c r="I27" s="56"/>
       <c r="J27" s="56"/>
       <c r="K27" s="56"/>
-      <c r="L27" s="58"/>
-      <c r="M27" s="58"/>
+      <c r="L27" s="56"/>
+      <c r="M27" s="56"/>
       <c r="N27" s="56"/>
-      <c r="O27" s="58" t="s">
-        <v>74</v>
-      </c>
-      <c r="P27" s="58"/>
-      <c r="Q27" s="58"/>
-      <c r="R27" s="58"/>
-      <c r="S27" s="58" t="s">
-        <v>75</v>
-      </c>
-      <c r="T27" s="58"/>
-      <c r="U27" s="58"/>
-      <c r="V27" s="58"/>
-      <c r="W27" s="58"/>
-      <c r="X27" s="58"/>
-      <c r="Y27" s="58" t="s">
-        <v>76</v>
-      </c>
-      <c r="Z27" s="58"/>
+      <c r="O27" s="56"/>
+      <c r="P27" s="56"/>
+      <c r="Q27" s="56"/>
+      <c r="R27" s="56"/>
+      <c r="S27" s="56"/>
+      <c r="T27" s="56"/>
+      <c r="U27" s="56"/>
+      <c r="V27" s="56"/>
+      <c r="W27" s="56"/>
+      <c r="X27" s="56"/>
+      <c r="Y27" s="56"/>
+      <c r="Z27" s="64"/>
       <c r="AA27" s="56"/>
-      <c r="AB27" s="58"/>
-      <c r="AC27" s="58"/>
-      <c r="AD27" s="58"/>
+      <c r="AB27" s="56"/>
+      <c r="AC27" s="56"/>
+      <c r="AD27" s="56"/>
       <c r="AE27" s="56"/>
       <c r="AF27" s="56"/>
       <c r="AG27" s="56"/>
-      <c r="AH27" s="58"/>
-    </row>
-    <row r="28" spans="1:34" ht="36" customHeight="1">
+      <c r="AH27" s="56"/>
+    </row>
+    <row r="28" spans="1:34" ht="14.25" customHeight="1">
       <c r="A28" s="56"/>
       <c r="B28" s="56"/>
       <c r="C28" s="57"/>
-      <c r="D28" s="58" t="s">
-        <v>77</v>
-      </c>
+      <c r="D28" s="58"/>
       <c r="E28" s="56"/>
       <c r="F28" s="56"/>
       <c r="G28" s="56"/>
@@ -6989,107 +7292,117 @@
       <c r="I28" s="56"/>
       <c r="J28" s="56"/>
       <c r="K28" s="56"/>
-      <c r="L28" s="58"/>
-      <c r="M28" s="58"/>
+      <c r="L28" s="56"/>
+      <c r="M28" s="56"/>
       <c r="N28" s="56"/>
-      <c r="O28" s="58" t="s">
-        <v>78</v>
-      </c>
-      <c r="P28" s="58"/>
-      <c r="Q28" s="58"/>
-      <c r="R28" s="58"/>
-      <c r="S28" s="58" t="s">
-        <v>79</v>
-      </c>
-      <c r="T28" s="58"/>
-      <c r="U28" s="58"/>
-      <c r="V28" s="58"/>
-      <c r="W28" s="58"/>
-      <c r="X28" s="58"/>
-      <c r="Y28" s="58" t="s">
-        <v>80</v>
-      </c>
-      <c r="Z28" s="59"/>
+      <c r="O28" s="56"/>
+      <c r="P28" s="56"/>
+      <c r="Q28" s="56"/>
+      <c r="R28" s="56"/>
+      <c r="S28" s="56"/>
+      <c r="T28" s="56"/>
+      <c r="U28" s="56"/>
+      <c r="V28" s="56"/>
+      <c r="W28" s="56"/>
+      <c r="X28" s="56"/>
+      <c r="Y28" s="56"/>
+      <c r="Z28" s="64"/>
       <c r="AA28" s="56"/>
-      <c r="AB28" s="58"/>
-      <c r="AC28" s="58"/>
-      <c r="AD28" s="58"/>
+      <c r="AB28" s="56"/>
+      <c r="AC28" s="56"/>
+      <c r="AD28" s="56"/>
       <c r="AE28" s="56"/>
       <c r="AF28" s="56"/>
       <c r="AG28" s="56"/>
-      <c r="AH28" s="58"/>
-    </row>
-    <row r="29" spans="1:34" ht="14.25" customHeight="1">
-      <c r="A29" s="22"/>
-      <c r="B29" s="22"/>
-      <c r="C29" s="23"/>
-      <c r="D29" s="22"/>
-      <c r="E29" s="22"/>
-      <c r="F29" s="24"/>
-      <c r="G29" s="24"/>
-      <c r="H29" s="24"/>
-      <c r="I29" s="24"/>
-      <c r="J29" s="24"/>
-      <c r="K29" s="24"/>
-      <c r="L29" s="22"/>
-      <c r="M29" s="22"/>
-      <c r="N29" s="22"/>
-      <c r="O29" s="22"/>
-      <c r="P29" s="22"/>
-      <c r="Q29" s="22"/>
-      <c r="R29" s="22"/>
-      <c r="S29" s="22"/>
-      <c r="T29" s="22"/>
-      <c r="U29" s="22"/>
-      <c r="V29" s="22"/>
-      <c r="W29" s="22"/>
-      <c r="X29" s="22"/>
-      <c r="Y29" s="22"/>
-      <c r="Z29" s="22"/>
-      <c r="AA29" s="22"/>
-      <c r="AB29" s="22"/>
-      <c r="AC29" s="22"/>
-      <c r="AD29" s="22"/>
-      <c r="AE29" s="22"/>
-      <c r="AF29" s="22"/>
-      <c r="AG29" s="22"/>
-      <c r="AH29" s="22"/>
-    </row>
-    <row r="30" spans="1:34" ht="14.25" customHeight="1">
-      <c r="A30" s="22"/>
-      <c r="B30" s="22"/>
-      <c r="C30" s="23"/>
-      <c r="D30" s="22"/>
-      <c r="E30" s="22"/>
-      <c r="F30" s="24"/>
-      <c r="G30" s="24"/>
-      <c r="H30" s="24"/>
-      <c r="I30" s="24"/>
-      <c r="J30" s="24"/>
-      <c r="K30" s="24"/>
-      <c r="L30" s="22"/>
-      <c r="M30" s="22"/>
-      <c r="N30" s="22"/>
-      <c r="O30" s="22"/>
-      <c r="P30" s="22"/>
-      <c r="Q30" s="22"/>
-      <c r="R30" s="22"/>
-      <c r="S30" s="22"/>
-      <c r="T30" s="22"/>
-      <c r="U30" s="22"/>
-      <c r="V30" s="22"/>
-      <c r="W30" s="22"/>
-      <c r="X30" s="22"/>
-      <c r="Y30" s="22"/>
-      <c r="Z30" s="22"/>
-      <c r="AA30" s="22"/>
-      <c r="AB30" s="22"/>
-      <c r="AC30" s="22"/>
-      <c r="AD30" s="22"/>
-      <c r="AE30" s="22"/>
-      <c r="AF30" s="22"/>
-      <c r="AG30" s="22"/>
-      <c r="AH30" s="22"/>
+      <c r="AH28" s="56"/>
+    </row>
+    <row r="29" spans="1:34" ht="33.75" customHeight="1">
+      <c r="A29" s="56"/>
+      <c r="B29" s="56"/>
+      <c r="C29" s="57"/>
+      <c r="D29" s="58" t="s">
+        <v>73</v>
+      </c>
+      <c r="E29" s="56"/>
+      <c r="F29" s="56"/>
+      <c r="G29" s="56"/>
+      <c r="H29" s="56"/>
+      <c r="I29" s="56"/>
+      <c r="J29" s="56"/>
+      <c r="K29" s="56"/>
+      <c r="L29" s="58"/>
+      <c r="M29" s="58"/>
+      <c r="N29" s="56"/>
+      <c r="O29" s="58" t="s">
+        <v>74</v>
+      </c>
+      <c r="P29" s="58"/>
+      <c r="Q29" s="58"/>
+      <c r="R29" s="58"/>
+      <c r="S29" s="58" t="s">
+        <v>75</v>
+      </c>
+      <c r="T29" s="58"/>
+      <c r="U29" s="58"/>
+      <c r="V29" s="58"/>
+      <c r="W29" s="58"/>
+      <c r="X29" s="58"/>
+      <c r="Y29" s="58" t="s">
+        <v>76</v>
+      </c>
+      <c r="Z29" s="58"/>
+      <c r="AA29" s="56"/>
+      <c r="AB29" s="58"/>
+      <c r="AC29" s="58"/>
+      <c r="AD29" s="58"/>
+      <c r="AE29" s="56"/>
+      <c r="AF29" s="56"/>
+      <c r="AG29" s="56"/>
+      <c r="AH29" s="58"/>
+    </row>
+    <row r="30" spans="1:34" ht="36" customHeight="1">
+      <c r="A30" s="56"/>
+      <c r="B30" s="56"/>
+      <c r="C30" s="57"/>
+      <c r="D30" s="58" t="s">
+        <v>77</v>
+      </c>
+      <c r="E30" s="56"/>
+      <c r="F30" s="56"/>
+      <c r="G30" s="56"/>
+      <c r="H30" s="56"/>
+      <c r="I30" s="56"/>
+      <c r="J30" s="56"/>
+      <c r="K30" s="56"/>
+      <c r="L30" s="58"/>
+      <c r="M30" s="58"/>
+      <c r="N30" s="56"/>
+      <c r="O30" s="58" t="s">
+        <v>78</v>
+      </c>
+      <c r="P30" s="58"/>
+      <c r="Q30" s="58"/>
+      <c r="R30" s="58"/>
+      <c r="S30" s="58" t="s">
+        <v>79</v>
+      </c>
+      <c r="T30" s="58"/>
+      <c r="U30" s="58"/>
+      <c r="V30" s="58"/>
+      <c r="W30" s="58"/>
+      <c r="X30" s="58"/>
+      <c r="Y30" s="58" t="s">
+        <v>80</v>
+      </c>
+      <c r="Z30" s="59"/>
+      <c r="AA30" s="56"/>
+      <c r="AB30" s="58"/>
+      <c r="AC30" s="58"/>
+      <c r="AD30" s="58"/>
+      <c r="AE30" s="56"/>
+      <c r="AF30" s="56"/>
+      <c r="AG30" s="56"/>
+      <c r="AH30" s="58"/>
     </row>
     <row r="31" spans="1:34" ht="14.25" customHeight="1">
       <c r="A31" s="22"/>
@@ -9611,9 +9924,81 @@
       <c r="AG100" s="22"/>
       <c r="AH100" s="22"/>
     </row>
+    <row r="101" spans="1:34" ht="14.25" customHeight="1">
+      <c r="A101" s="22"/>
+      <c r="B101" s="22"/>
+      <c r="C101" s="23"/>
+      <c r="D101" s="22"/>
+      <c r="E101" s="22"/>
+      <c r="F101" s="24"/>
+      <c r="G101" s="24"/>
+      <c r="H101" s="24"/>
+      <c r="I101" s="24"/>
+      <c r="J101" s="24"/>
+      <c r="K101" s="24"/>
+      <c r="L101" s="22"/>
+      <c r="M101" s="22"/>
+      <c r="N101" s="22"/>
+      <c r="O101" s="22"/>
+      <c r="P101" s="22"/>
+      <c r="Q101" s="22"/>
+      <c r="R101" s="22"/>
+      <c r="S101" s="22"/>
+      <c r="T101" s="22"/>
+      <c r="U101" s="22"/>
+      <c r="V101" s="22"/>
+      <c r="W101" s="22"/>
+      <c r="X101" s="22"/>
+      <c r="Y101" s="22"/>
+      <c r="Z101" s="22"/>
+      <c r="AA101" s="22"/>
+      <c r="AB101" s="22"/>
+      <c r="AC101" s="22"/>
+      <c r="AD101" s="22"/>
+      <c r="AE101" s="22"/>
+      <c r="AF101" s="22"/>
+      <c r="AG101" s="22"/>
+      <c r="AH101" s="22"/>
+    </row>
+    <row r="102" spans="1:34" ht="14.25" customHeight="1">
+      <c r="A102" s="22"/>
+      <c r="B102" s="22"/>
+      <c r="C102" s="23"/>
+      <c r="D102" s="22"/>
+      <c r="E102" s="22"/>
+      <c r="F102" s="24"/>
+      <c r="G102" s="24"/>
+      <c r="H102" s="24"/>
+      <c r="I102" s="24"/>
+      <c r="J102" s="24"/>
+      <c r="K102" s="24"/>
+      <c r="L102" s="22"/>
+      <c r="M102" s="22"/>
+      <c r="N102" s="22"/>
+      <c r="O102" s="22"/>
+      <c r="P102" s="22"/>
+      <c r="Q102" s="22"/>
+      <c r="R102" s="22"/>
+      <c r="S102" s="22"/>
+      <c r="T102" s="22"/>
+      <c r="U102" s="22"/>
+      <c r="V102" s="22"/>
+      <c r="W102" s="22"/>
+      <c r="X102" s="22"/>
+      <c r="Y102" s="22"/>
+      <c r="Z102" s="22"/>
+      <c r="AA102" s="22"/>
+      <c r="AB102" s="22"/>
+      <c r="AC102" s="22"/>
+      <c r="AD102" s="22"/>
+      <c r="AE102" s="22"/>
+      <c r="AF102" s="22"/>
+      <c r="AG102" s="22"/>
+      <c r="AH102" s="22"/>
+    </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="B16:K16"/>
+    <mergeCell ref="B18:K18"/>
   </mergeCells>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup paperSize="9" orientation="portrait"/>

</xml_diff>

<commit_message>
update FINAL.xlsx with revised profit-sharing calculations
</commit_message>
<xml_diff>
--- a/FINAL.xlsx
+++ b/FINAL.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Lenovo\bagi-hasil\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A3E5AE62-8701-4ED0-A08B-1814EE8E995C}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{500FB25A-A9A9-41D0-8F0D-493EBF6D4A89}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2332,63 +2332,63 @@
       </c>
       <c r="B15" s="19"/>
       <c r="C15" s="20">
-        <f>SUM(C5:C14)</f>
+        <f t="shared" ref="C15:Q15" si="22">SUM(C5:C14)</f>
         <v>584</v>
       </c>
       <c r="D15" s="20">
-        <f>SUM(D5:D14)</f>
+        <f t="shared" si="22"/>
         <v>73429250</v>
       </c>
       <c r="E15" s="20">
-        <f>SUM(E5:E14)</f>
+        <f t="shared" si="22"/>
         <v>62847500</v>
       </c>
       <c r="F15" s="20">
-        <f>SUM(F5:F14)</f>
+        <f t="shared" si="22"/>
         <v>20319000</v>
       </c>
       <c r="G15" s="20">
-        <f>SUM(G5:G14)</f>
+        <f t="shared" si="22"/>
         <v>0</v>
       </c>
       <c r="H15" s="20">
-        <f>SUM(H5:H14)</f>
+        <f t="shared" si="22"/>
         <v>9458000</v>
       </c>
       <c r="I15" s="20">
-        <f>SUM(I5:I14)</f>
+        <f t="shared" si="22"/>
         <v>166053750</v>
       </c>
       <c r="J15" s="20">
-        <f>SUM(J5:J14)</f>
+        <f t="shared" si="22"/>
         <v>14685850</v>
       </c>
       <c r="K15" s="20">
-        <f>SUM(K5:K14)</f>
+        <f t="shared" si="22"/>
         <v>19455895</v>
       </c>
       <c r="L15" s="20">
-        <f>SUM(L5:L14)</f>
+        <f t="shared" si="22"/>
         <v>6802875</v>
       </c>
       <c r="M15" s="20">
-        <f>SUM(M5:M14)</f>
+        <f t="shared" si="22"/>
         <v>0</v>
       </c>
       <c r="N15" s="20">
-        <f>SUM(N5:N14)</f>
+        <f t="shared" si="22"/>
         <v>2837400</v>
       </c>
       <c r="O15" s="20">
-        <f>SUM(O5:O14)</f>
+        <f t="shared" si="22"/>
         <v>43782020</v>
       </c>
       <c r="P15" s="20">
-        <f>SUM(P5:P14)</f>
+        <f t="shared" si="22"/>
         <v>49816125</v>
       </c>
       <c r="Q15" s="20">
-        <f>SUM(Q5:Q14)</f>
+        <f t="shared" si="22"/>
         <v>-6034105</v>
       </c>
       <c r="R15" s="21">
@@ -2396,63 +2396,63 @@
         <v>26.366173603426603</v>
       </c>
       <c r="S15" s="20">
-        <f t="shared" ref="S15:AG15" si="22">SUM(S5:S14)</f>
+        <f t="shared" ref="S15:AG15" si="23">SUM(S5:S14)</f>
         <v>396300</v>
       </c>
       <c r="T15" s="20">
-        <f t="shared" si="22"/>
+        <f t="shared" si="23"/>
         <v>0</v>
       </c>
       <c r="U15" s="20">
-        <f t="shared" si="22"/>
+        <f t="shared" si="23"/>
         <v>343805</v>
       </c>
       <c r="V15" s="20">
-        <f t="shared" si="22"/>
+        <f t="shared" si="23"/>
         <v>0</v>
       </c>
       <c r="W15" s="20">
-        <f t="shared" si="22"/>
+        <f t="shared" si="23"/>
         <v>0</v>
       </c>
       <c r="X15" s="20">
-        <f t="shared" si="22"/>
+        <f t="shared" si="23"/>
         <v>0</v>
       </c>
       <c r="Y15" s="20">
-        <f t="shared" si="22"/>
+        <f t="shared" si="23"/>
         <v>30000</v>
       </c>
       <c r="Z15" s="20">
-        <f t="shared" si="22"/>
+        <f t="shared" si="23"/>
         <v>100000</v>
       </c>
       <c r="AA15" s="20">
-        <f t="shared" si="22"/>
+        <f t="shared" si="23"/>
         <v>500000</v>
       </c>
       <c r="AB15" s="20">
-        <f t="shared" si="22"/>
+        <f t="shared" si="23"/>
         <v>1370105</v>
       </c>
       <c r="AC15" s="20">
-        <f t="shared" si="22"/>
+        <f t="shared" si="23"/>
         <v>0</v>
       </c>
       <c r="AD15" s="20">
-        <f t="shared" si="22"/>
+        <f t="shared" si="23"/>
         <v>42411915</v>
       </c>
       <c r="AE15" s="20">
-        <f t="shared" si="22"/>
+        <f t="shared" si="23"/>
         <v>1165600</v>
       </c>
       <c r="AF15" s="20">
-        <f t="shared" si="22"/>
+        <f t="shared" si="23"/>
         <v>51560605.149999999</v>
       </c>
       <c r="AG15" s="20">
-        <f t="shared" si="22"/>
+        <f t="shared" si="23"/>
         <v>52726205.149999999</v>
       </c>
     </row>
@@ -5892,7 +5892,7 @@
         <v>0</v>
       </c>
       <c r="O8" s="47">
-        <f t="shared" ref="O8:O17" si="1">SUM(M8:N8)</f>
+        <f t="shared" ref="O8" si="1">SUM(M8:N8)</f>
         <v>10714040</v>
       </c>
       <c r="P8" s="47">
@@ -5936,11 +5936,11 @@
         <v>100000</v>
       </c>
       <c r="Z8" s="47">
-        <f t="shared" ref="Z8:Z17" si="2">O8-Y8</f>
+        <f t="shared" ref="Z8" si="2">O8-Y8</f>
         <v>10614040</v>
       </c>
       <c r="AA8" s="48" t="e">
-        <f t="shared" ref="AA8:AA17" ca="1" si="3">_xludf.TEXTJOIN(" | ",TRUE,IF(V8&gt;0,"Biaya Pendaftaran Koperasi: "&amp;TEXT(V8,"#.##0"),""),IF(W8&gt;0,"Simpanan Pokok: "&amp;TEXT(W8,"#.##0"),""),IF(X8&gt;0,"Simpanan Wajib: "&amp;TEXT(X8,"#.##0"),""))</f>
+        <f t="shared" ref="AA8" ca="1" si="3">_xludf.TEXTJOIN(" | ",TRUE,IF(V8&gt;0,"Biaya Pendaftaran Koperasi: "&amp;TEXT(V8,"#.##0"),""),IF(W8&gt;0,"Simpanan Pokok: "&amp;TEXT(W8,"#.##0"),""),IF(X8&gt;0,"Simpanan Wajib: "&amp;TEXT(X8,"#.##0"),""))</f>
         <v>#NAME?</v>
       </c>
       <c r="AB8" s="41"/>
@@ -5974,7 +5974,7 @@
       <c r="H9" s="42"/>
       <c r="I9" s="45"/>
       <c r="J9" s="42" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" ref="J9:J17" si="4">CONCATENATE($G$7,G9,$H$7,H9,$I$7,I9)</f>
         <v xml:space="preserve">Bank BSI No. Rek.  A/n </v>
       </c>
       <c r="K9" s="42" t="s">
@@ -5993,7 +5993,7 @@
         <v>0</v>
       </c>
       <c r="O9" s="47">
-        <f t="shared" ref="O9:O17" si="4">SUM(M9:N9)</f>
+        <f t="shared" ref="O9:O17" si="5">SUM(M9:N9)</f>
         <v>10252520</v>
       </c>
       <c r="P9" s="47">
@@ -6037,11 +6037,11 @@
         <v>443805</v>
       </c>
       <c r="Z9" s="47">
-        <f t="shared" ref="Z9:Z17" si="5">O9-Y9</f>
+        <f t="shared" ref="Z9:Z17" si="6">O9-Y9</f>
         <v>9808715</v>
       </c>
       <c r="AA9" s="48" t="e">
-        <f t="shared" ref="AA9:AA17" ca="1" si="6">_xludf.TEXTJOIN(" | ",TRUE,IF(V9&gt;0,"Biaya Pendaftaran Koperasi: "&amp;TEXT(V9,"#.##0"),""),IF(W9&gt;0,"Simpanan Pokok: "&amp;TEXT(W9,"#.##0"),""),IF(X9&gt;0,"Simpanan Wajib: "&amp;TEXT(X9,"#.##0"),""))</f>
+        <f t="shared" ref="AA9:AA17" ca="1" si="7">_xludf.TEXTJOIN(" | ",TRUE,IF(V9&gt;0,"Biaya Pendaftaran Koperasi: "&amp;TEXT(V9,"#.##0"),""),IF(W9&gt;0,"Simpanan Pokok: "&amp;TEXT(W9,"#.##0"),""),IF(X9&gt;0,"Simpanan Wajib: "&amp;TEXT(X9,"#.##0"),""))</f>
         <v>#NAME?</v>
       </c>
       <c r="AB9" s="41"/>
@@ -6075,7 +6075,7 @@
       <c r="H10" s="42"/>
       <c r="I10" s="45"/>
       <c r="J10" s="42" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="4"/>
         <v xml:space="preserve">Bank BSI No. Rek.  A/n </v>
       </c>
       <c r="K10" s="42" t="s">
@@ -6094,7 +6094,7 @@
         <v>0</v>
       </c>
       <c r="O10" s="47">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>8265240</v>
       </c>
       <c r="P10" s="47">
@@ -6138,11 +6138,11 @@
         <v>184300</v>
       </c>
       <c r="Z10" s="47">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>8080940</v>
       </c>
       <c r="AA10" s="48" t="e">
-        <f t="shared" ca="1" si="6"/>
+        <f t="shared" ca="1" si="7"/>
         <v>#NAME?</v>
       </c>
       <c r="AB10" s="41"/>
@@ -6176,7 +6176,7 @@
       <c r="H11" s="42"/>
       <c r="I11" s="45"/>
       <c r="J11" s="42" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="4"/>
         <v xml:space="preserve">Bank BSI No. Rek.  A/n </v>
       </c>
       <c r="K11" s="42" t="s">
@@ -6195,7 +6195,7 @@
         <v>0</v>
       </c>
       <c r="O11" s="47">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>5870920</v>
       </c>
       <c r="P11" s="47">
@@ -6239,11 +6239,11 @@
         <v>160000</v>
       </c>
       <c r="Z11" s="47">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>5710920</v>
       </c>
       <c r="AA11" s="48" t="e">
-        <f t="shared" ca="1" si="6"/>
+        <f t="shared" ca="1" si="7"/>
         <v>#NAME?</v>
       </c>
       <c r="AB11" s="41"/>
@@ -6275,9 +6275,9 @@
         <v>68</v>
       </c>
       <c r="H12" s="42"/>
-      <c r="I12" s="44"/>
+      <c r="I12" s="45"/>
       <c r="J12" s="42" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="4"/>
         <v xml:space="preserve">Bank BSI No. Rek.  A/n </v>
       </c>
       <c r="K12" s="42" t="s">
@@ -6296,7 +6296,7 @@
         <v>0</v>
       </c>
       <c r="O12" s="47">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>4266200</v>
       </c>
       <c r="P12" s="47">
@@ -6340,11 +6340,11 @@
         <v>157000</v>
       </c>
       <c r="Z12" s="47">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>4109200</v>
       </c>
       <c r="AA12" s="48" t="e">
-        <f t="shared" ca="1" si="6"/>
+        <f t="shared" ca="1" si="7"/>
         <v>#NAME?</v>
       </c>
       <c r="AB12" s="41"/>
@@ -6378,7 +6378,7 @@
       <c r="H13" s="42"/>
       <c r="I13" s="45"/>
       <c r="J13" s="42" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="4"/>
         <v xml:space="preserve">Bank BSI No. Rek.  A/n </v>
       </c>
       <c r="K13" s="42" t="s">
@@ -6397,7 +6397,7 @@
         <v>0</v>
       </c>
       <c r="O13" s="47">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>4154500</v>
       </c>
       <c r="P13" s="47">
@@ -6441,11 +6441,11 @@
         <v>220000</v>
       </c>
       <c r="Z13" s="47">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>3934500</v>
       </c>
       <c r="AA13" s="48" t="e">
-        <f t="shared" ca="1" si="6"/>
+        <f t="shared" ca="1" si="7"/>
         <v>#NAME?</v>
       </c>
       <c r="AB13" s="41"/>
@@ -6479,7 +6479,7 @@
       <c r="H14" s="42"/>
       <c r="I14" s="45"/>
       <c r="J14" s="42" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="4"/>
         <v xml:space="preserve">Bank BSI No. Rek.  A/n </v>
       </c>
       <c r="K14" s="42" t="s">
@@ -6498,7 +6498,7 @@
         <v>0</v>
       </c>
       <c r="O14" s="47">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>99300</v>
       </c>
       <c r="P14" s="47">
@@ -6542,11 +6542,11 @@
         <v>52500</v>
       </c>
       <c r="Z14" s="47">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>46800</v>
       </c>
       <c r="AA14" s="48" t="e">
-        <f t="shared" ca="1" si="6"/>
+        <f t="shared" ca="1" si="7"/>
         <v>#NAME?</v>
       </c>
       <c r="AB14" s="41"/>
@@ -6578,9 +6578,9 @@
         <v>68</v>
       </c>
       <c r="H15" s="42"/>
-      <c r="I15" s="44"/>
+      <c r="I15" s="45"/>
       <c r="J15" s="42" t="str">
-        <f t="shared" ref="J15" si="7">CONCATENATE($G$7,G15,$H$7,H15,$I$7,I15)</f>
+        <f t="shared" si="4"/>
         <v xml:space="preserve">Bank BSI No. Rek.  A/n </v>
       </c>
       <c r="K15" s="42" t="s">
@@ -6599,7 +6599,7 @@
         <v>0</v>
       </c>
       <c r="O15" s="47">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>30000</v>
       </c>
       <c r="P15" s="47">
@@ -6643,11 +6643,11 @@
         <v>0</v>
       </c>
       <c r="Z15" s="47">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>30000</v>
       </c>
       <c r="AA15" s="48" t="e">
-        <f t="shared" ca="1" si="6"/>
+        <f t="shared" ca="1" si="7"/>
         <v>#NAME?</v>
       </c>
       <c r="AB15" s="41"/>
@@ -6679,9 +6679,9 @@
         <v>68</v>
       </c>
       <c r="H16" s="42"/>
-      <c r="I16" s="44"/>
+      <c r="I16" s="45"/>
       <c r="J16" s="42" t="str">
-        <f t="shared" ref="J16" si="8">CONCATENATE($G$7,G16,$H$7,H16,$I$7,I16)</f>
+        <f t="shared" si="4"/>
         <v xml:space="preserve">Bank BSI No. Rek.  A/n </v>
       </c>
       <c r="K16" s="42" t="s">
@@ -6700,7 +6700,7 @@
         <v>0</v>
       </c>
       <c r="O16" s="47">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>99300</v>
       </c>
       <c r="P16" s="47">
@@ -6744,11 +6744,11 @@
         <v>52500</v>
       </c>
       <c r="Z16" s="47">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>46800</v>
       </c>
       <c r="AA16" s="48" t="e">
-        <f t="shared" ca="1" si="6"/>
+        <f t="shared" ca="1" si="7"/>
         <v>#NAME?</v>
       </c>
       <c r="AB16" s="41"/>
@@ -6780,9 +6780,9 @@
         <v>68</v>
       </c>
       <c r="H17" s="42"/>
-      <c r="I17" s="44"/>
+      <c r="I17" s="45"/>
       <c r="J17" s="42" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="4"/>
         <v xml:space="preserve">Bank BSI No. Rek.  A/n </v>
       </c>
       <c r="K17" s="42" t="s">
@@ -6801,7 +6801,7 @@
         <v>0</v>
       </c>
       <c r="O17" s="47">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>30000</v>
       </c>
       <c r="P17" s="47">
@@ -6845,11 +6845,11 @@
         <v>0</v>
       </c>
       <c r="Z17" s="47">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>30000</v>
       </c>
       <c r="AA17" s="48" t="e">
-        <f t="shared" ca="1" si="6"/>
+        <f t="shared" ca="1" si="7"/>
         <v>#NAME?</v>
       </c>
       <c r="AB17" s="41"/>
@@ -6875,63 +6875,63 @@
       <c r="J18" s="66"/>
       <c r="K18" s="67"/>
       <c r="L18" s="50">
-        <f t="shared" ref="L18:Z18" si="9">SUM(L8:L17)</f>
+        <f t="shared" ref="L18:Z18" si="8">SUM(L8:L17)</f>
         <v>166053750</v>
       </c>
       <c r="M18" s="50">
-        <f t="shared" si="9"/>
+        <f t="shared" si="8"/>
         <v>43782020</v>
       </c>
       <c r="N18" s="50">
-        <f t="shared" si="9"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="O18" s="50">
-        <f t="shared" si="9"/>
+        <f t="shared" si="8"/>
         <v>43782020</v>
       </c>
       <c r="P18" s="50">
-        <f t="shared" si="9"/>
+        <f t="shared" si="8"/>
         <v>396300</v>
       </c>
       <c r="Q18" s="50">
-        <f t="shared" si="9"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="R18" s="50">
-        <f t="shared" si="9"/>
+        <f t="shared" si="8"/>
         <v>343805</v>
       </c>
       <c r="S18" s="50">
-        <f t="shared" si="9"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="T18" s="50">
-        <f t="shared" si="9"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="U18" s="50">
-        <f t="shared" si="9"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="V18" s="50">
-        <f t="shared" si="9"/>
+        <f t="shared" si="8"/>
         <v>30000</v>
       </c>
       <c r="W18" s="50">
-        <f t="shared" si="9"/>
+        <f t="shared" si="8"/>
         <v>100000</v>
       </c>
       <c r="X18" s="50">
-        <f t="shared" si="9"/>
+        <f t="shared" si="8"/>
         <v>500000</v>
       </c>
       <c r="Y18" s="50">
-        <f t="shared" si="9"/>
+        <f t="shared" si="8"/>
         <v>1370105</v>
       </c>
       <c r="Z18" s="50">
-        <f t="shared" si="9"/>
+        <f t="shared" si="8"/>
         <v>42411915</v>
       </c>
       <c r="AA18" s="51"/>

</xml_diff>